<commit_message>
Sync planning SharePoint : S34
</commit_message>
<xml_diff>
--- a/Plannings 2026 S34.xlsx
+++ b/Plannings 2026 S34.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cdalpes.sharepoint.com/sites/msteams_bd0f90/Documents partages/02. USP - TOS - General/RH/Plannings/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{559C6429-F12D-441A-BD84-FBDC171A605E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="2" documentId="8_{559C6429-F12D-441A-BD84-FBDC171A605E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F5845C06-B34D-4CFD-B82C-4A1429626F94}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="238" uniqueCount="84">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="236" uniqueCount="83">
   <si>
     <t>Planning des salariés du 17/08/2026 au 23/08/2026</t>
   </si>
@@ -179,9 +179,6 @@
   </si>
   <si>
     <t>DOVINA Théo</t>
-  </si>
-  <si>
-    <t>20:00/24:00</t>
   </si>
   <si>
     <t>19:00/24:00</t>
@@ -2996,50 +2993,6 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>3</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>34</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>3</xdr:col>
-      <xdr:colOff>123825</xdr:colOff>
-      <xdr:row>34</xdr:row>
-      <xdr:rowOff>123825</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="51" name="Picture 1" descr="Picture">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000033000000}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="0" y="0"/>
-          <a:ext cx="123825" cy="123825"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
       <xdr:col>4</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>34</xdr:row>
@@ -4672,7 +4625,7 @@
     </row>
     <row r="3" spans="1:8" s="43" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B3" s="44" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="C3" s="44"/>
       <c r="D3" s="44"/>
@@ -4950,7 +4903,7 @@
         <v>33</v>
       </c>
       <c r="B20" s="31" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C20" s="32"/>
       <c r="D20" s="32"/>
@@ -5229,9 +5182,7 @@
       </c>
       <c r="B35" s="18"/>
       <c r="C35" s="18"/>
-      <c r="D35" s="18" t="s">
-        <v>12</v>
-      </c>
+      <c r="D35" s="18"/>
       <c r="E35" s="18" t="s">
         <v>12</v>
       </c>
@@ -5245,11 +5196,9 @@
       <c r="A36" s="20"/>
       <c r="B36" s="22"/>
       <c r="C36" s="22"/>
-      <c r="D36" s="22" t="s">
+      <c r="D36" s="22"/>
+      <c r="E36" s="22" t="s">
         <v>48</v>
-      </c>
-      <c r="E36" s="22" t="s">
-        <v>49</v>
       </c>
       <c r="F36" s="22" t="s">
         <v>44</v>
@@ -5259,7 +5208,7 @@
     </row>
     <row r="37" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A37" s="24" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B37" s="25"/>
       <c r="C37" s="26"/>
@@ -5271,7 +5220,7 @@
     </row>
     <row r="38" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A38" s="24" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B38" s="25"/>
       <c r="C38" s="26"/>
@@ -5283,7 +5232,7 @@
     </row>
     <row r="39" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A39" s="30" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B39" s="31"/>
       <c r="C39" s="32"/>
@@ -5295,7 +5244,7 @@
     </row>
     <row r="40" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A40" s="16" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B40" s="37" t="s">
         <v>17</v>
@@ -5398,19 +5347,19 @@
     <row r="45" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A45" s="28"/>
       <c r="B45" s="38" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C45" s="38" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="D45" s="38" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="E45" s="38" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F45" s="38" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="G45" s="1"/>
       <c r="H45" s="29"/>
@@ -5517,7 +5466,7 @@
     </row>
     <row r="52" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A52" s="24" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B52" s="25"/>
       <c r="C52" s="26"/>
@@ -5529,7 +5478,7 @@
     </row>
     <row r="53" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A53" s="24" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B53" s="25"/>
       <c r="C53" s="26"/>
@@ -5541,7 +5490,7 @@
     </row>
     <row r="54" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A54" s="24" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B54" s="25"/>
       <c r="C54" s="26"/>
@@ -5553,7 +5502,7 @@
     </row>
     <row r="55" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A55" s="16" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B55" s="18"/>
       <c r="C55" s="18"/>
@@ -5574,12 +5523,12 @@
       <c r="F56" s="22"/>
       <c r="G56" s="22"/>
       <c r="H56" s="23" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="57" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A57" s="24" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B57" s="25"/>
       <c r="C57" s="26"/>
@@ -5591,7 +5540,7 @@
     </row>
     <row r="58" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A58" s="24" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B58" s="25"/>
       <c r="C58" s="26"/>
@@ -5603,10 +5552,10 @@
     </row>
     <row r="59" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A59" s="24" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B59" s="25" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C59" s="26"/>
       <c r="D59" s="26"/>
@@ -5617,7 +5566,7 @@
     </row>
     <row r="60" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A60" s="24" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B60" s="25"/>
       <c r="C60" s="26"/>
@@ -5629,7 +5578,7 @@
     </row>
     <row r="61" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A61" s="24" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B61" s="25"/>
       <c r="C61" s="26"/>
@@ -5641,7 +5590,7 @@
     </row>
     <row r="62" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A62" s="24" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B62" s="25"/>
       <c r="C62" s="26"/>
@@ -5653,7 +5602,7 @@
     </row>
     <row r="63" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A63" s="24" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B63" s="25"/>
       <c r="C63" s="26"/>
@@ -5722,7 +5671,7 @@
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B4" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C4" s="13"/>
       <c r="D4" s="13"/>
@@ -5730,7 +5679,7 @@
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B5" s="14" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C5" s="14"/>
       <c r="D5" s="14"/>
@@ -5741,16 +5690,16 @@
         <v>3</v>
       </c>
       <c r="B6" s="6" t="s">
+        <v>69</v>
+      </c>
+      <c r="C6" s="6" t="s">
         <v>70</v>
       </c>
-      <c r="C6" s="6" t="s">
+      <c r="D6" s="6" t="s">
         <v>71</v>
       </c>
-      <c r="D6" s="6" t="s">
+      <c r="E6" s="6" t="s">
         <v>72</v>
-      </c>
-      <c r="E6" s="6" t="s">
-        <v>73</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
@@ -5925,7 +5874,7 @@
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" s="5" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B17" s="7">
         <v>0</v>
@@ -5942,7 +5891,7 @@
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" s="5" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B18" s="7">
         <v>0</v>
@@ -5959,7 +5908,7 @@
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" s="5" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B19" s="7">
         <v>0</v>
@@ -5976,7 +5925,7 @@
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" s="5" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B20" s="7">
         <v>0</v>
@@ -5993,7 +5942,7 @@
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" s="5" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B21" s="7">
         <v>0</v>
@@ -6010,7 +5959,7 @@
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" s="5" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B22" s="7">
         <v>0</v>
@@ -6027,7 +5976,7 @@
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" s="5" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B23" s="7">
         <v>0</v>
@@ -6044,7 +5993,7 @@
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" s="5" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B24" s="7">
         <v>0</v>
@@ -6061,7 +6010,7 @@
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" s="5" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B25" s="7">
         <v>0</v>
@@ -6078,7 +6027,7 @@
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" s="5" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B26" s="7">
         <v>0</v>
@@ -6095,7 +6044,7 @@
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" s="5" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B27" s="7">
         <v>0</v>
@@ -6112,7 +6061,7 @@
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28" s="5" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B28" s="7">
         <v>0</v>
@@ -6129,7 +6078,7 @@
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29" s="5" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B29" s="7">
         <v>0</v>
@@ -6146,7 +6095,7 @@
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A30" s="5" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B30" s="7">
         <v>0</v>
@@ -6163,7 +6112,7 @@
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A31" s="5" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B31" s="7">
         <v>0</v>
@@ -6180,7 +6129,7 @@
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A32" s="5" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B32" s="7">
         <v>0</v>
@@ -6230,40 +6179,40 @@
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="10" t="s">
+        <v>73</v>
+      </c>
+      <c r="B4" s="11" t="s">
         <v>74</v>
-      </c>
-      <c r="B4" s="11" t="s">
-        <v>75</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="10" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B5" s="11"/>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="10" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B6" s="11" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="B7" s="11" t="s">
         <v>78</v>
-      </c>
-      <c r="B7" s="11" t="s">
-        <v>79</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" s="10" t="s">
+        <v>79</v>
+      </c>
+      <c r="B8" s="11" t="s">
         <v>80</v>
-      </c>
-      <c r="B8" s="11" t="s">
-        <v>81</v>
       </c>
     </row>
   </sheetData>
@@ -6444,13 +6393,13 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B5C027A0-44BD-4A75-841B-07F4C346E0F4}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A1C2E62D-B5C2-4797-8435-153EB3ADEDA3}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{67EC5373-55CE-4190-A766-361458A103D5}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{776D5F97-2FA8-4677-BB70-78096B3628DE}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C3BC4490-B2FC-4F13-B0AE-74C335B88878}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DBF84BC3-7FCF-4F2C-B2F1-F8A377E9AC78}"/>
 </file>
</xml_diff>